<commit_message>
Add OpenRouter API To GPT LLM for query
</commit_message>
<xml_diff>
--- a/Excels/customers_export.xlsx
+++ b/Excels/customers_export.xlsx
@@ -212,7 +212,7 @@
       </c>
       <c r="X2" s="0" t="inlineStr">
         <is>
-          <t>537000.00</t>
+          <t>1640000.00</t>
         </is>
       </c>
       <c r="Z2" s="0" t="inlineStr">
@@ -244,7 +244,7 @@
       </c>
       <c r="X3" s="0" t="inlineStr">
         <is>
-          <t>1876100.00</t>
+          <t>1944100.00</t>
         </is>
       </c>
       <c r="Z3" s="0" t="inlineStr">
@@ -308,7 +308,7 @@
       </c>
       <c r="X5" s="0" t="inlineStr">
         <is>
-          <t>957500.00</t>
+          <t>1743500.00</t>
         </is>
       </c>
       <c r="Z5" s="0" t="inlineStr">
@@ -340,7 +340,7 @@
       </c>
       <c r="X6" s="0" t="inlineStr">
         <is>
-          <t>2014500.00</t>
+          <t>2895000.00</t>
         </is>
       </c>
       <c r="Z6" s="0" t="inlineStr">
@@ -404,7 +404,7 @@
       </c>
       <c r="X8" s="0" t="inlineStr">
         <is>
-          <t>345500.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z8" s="0" t="inlineStr">
@@ -500,7 +500,7 @@
       </c>
       <c r="X11" s="0" t="inlineStr">
         <is>
-          <t>1597000.00</t>
+          <t>1477000.00</t>
         </is>
       </c>
       <c r="Z11" s="0" t="inlineStr">
@@ -532,7 +532,7 @@
       </c>
       <c r="X12" s="0" t="inlineStr">
         <is>
-          <t>16364300.00</t>
+          <t>29980500.00</t>
         </is>
       </c>
       <c r="Z12" s="0" t="inlineStr">
@@ -884,7 +884,7 @@
       </c>
       <c r="X23" s="0" t="inlineStr">
         <is>
-          <t>796000.00</t>
+          <t>1941000.00</t>
         </is>
       </c>
       <c r="Z23" s="0" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="X24" s="0" t="inlineStr">
         <is>
-          <t>1533000.00</t>
+          <t>2526000.00</t>
         </is>
       </c>
       <c r="Z24" s="0" t="inlineStr">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="X28" s="0" t="inlineStr">
         <is>
-          <t>1341000.00</t>
+          <t>1778000.00</t>
         </is>
       </c>
       <c r="Z28" s="0" t="inlineStr">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="X29" s="0" t="inlineStr">
         <is>
-          <t>263000.00</t>
+          <t>653000.00</t>
         </is>
       </c>
       <c r="Z29" s="0" t="inlineStr">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="X30" s="0" t="inlineStr">
         <is>
-          <t>350000.00</t>
+          <t>410000.00</t>
         </is>
       </c>
       <c r="Z30" s="0" t="inlineStr">
@@ -1140,7 +1140,7 @@
       </c>
       <c r="X31" s="0" t="inlineStr">
         <is>
-          <t>267000.00</t>
+          <t>637000.00</t>
         </is>
       </c>
       <c r="Z31" s="0" t="inlineStr">
@@ -1556,7 +1556,7 @@
       </c>
       <c r="X44" s="0" t="inlineStr">
         <is>
-          <t>68000.00</t>
+          <t>408000.00</t>
         </is>
       </c>
       <c r="Z44" s="0" t="inlineStr">
@@ -1716,7 +1716,7 @@
       </c>
       <c r="X49" s="0" t="inlineStr">
         <is>
-          <t>684000.00</t>
+          <t>1020000.00</t>
         </is>
       </c>
       <c r="Z49" s="0" t="inlineStr">
@@ -1812,7 +1812,7 @@
       </c>
       <c r="X52" s="0" t="inlineStr">
         <is>
-          <t>730000.00</t>
+          <t>1198000.00</t>
         </is>
       </c>
       <c r="Z52" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Revert "Add OpenRouter API To GPT LLM for query"
This reverts commit fbc835ac77f0f81116c672353472f942aff5e02f.
</commit_message>
<xml_diff>
--- a/Excels/customers_export.xlsx
+++ b/Excels/customers_export.xlsx
@@ -212,7 +212,7 @@
       </c>
       <c r="X2" s="0" t="inlineStr">
         <is>
-          <t>1640000.00</t>
+          <t>537000.00</t>
         </is>
       </c>
       <c r="Z2" s="0" t="inlineStr">
@@ -244,7 +244,7 @@
       </c>
       <c r="X3" s="0" t="inlineStr">
         <is>
-          <t>1944100.00</t>
+          <t>1876100.00</t>
         </is>
       </c>
       <c r="Z3" s="0" t="inlineStr">
@@ -308,7 +308,7 @@
       </c>
       <c r="X5" s="0" t="inlineStr">
         <is>
-          <t>1743500.00</t>
+          <t>957500.00</t>
         </is>
       </c>
       <c r="Z5" s="0" t="inlineStr">
@@ -340,7 +340,7 @@
       </c>
       <c r="X6" s="0" t="inlineStr">
         <is>
-          <t>2895000.00</t>
+          <t>2014500.00</t>
         </is>
       </c>
       <c r="Z6" s="0" t="inlineStr">
@@ -404,7 +404,7 @@
       </c>
       <c r="X8" s="0" t="inlineStr">
         <is>
-          <t>0.00</t>
+          <t>345500.00</t>
         </is>
       </c>
       <c r="Z8" s="0" t="inlineStr">
@@ -500,7 +500,7 @@
       </c>
       <c r="X11" s="0" t="inlineStr">
         <is>
-          <t>1477000.00</t>
+          <t>1597000.00</t>
         </is>
       </c>
       <c r="Z11" s="0" t="inlineStr">
@@ -532,7 +532,7 @@
       </c>
       <c r="X12" s="0" t="inlineStr">
         <is>
-          <t>29980500.00</t>
+          <t>16364300.00</t>
         </is>
       </c>
       <c r="Z12" s="0" t="inlineStr">
@@ -884,7 +884,7 @@
       </c>
       <c r="X23" s="0" t="inlineStr">
         <is>
-          <t>1941000.00</t>
+          <t>796000.00</t>
         </is>
       </c>
       <c r="Z23" s="0" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="X24" s="0" t="inlineStr">
         <is>
-          <t>2526000.00</t>
+          <t>1533000.00</t>
         </is>
       </c>
       <c r="Z24" s="0" t="inlineStr">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="X28" s="0" t="inlineStr">
         <is>
-          <t>1778000.00</t>
+          <t>1341000.00</t>
         </is>
       </c>
       <c r="Z28" s="0" t="inlineStr">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="X29" s="0" t="inlineStr">
         <is>
-          <t>653000.00</t>
+          <t>263000.00</t>
         </is>
       </c>
       <c r="Z29" s="0" t="inlineStr">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="X30" s="0" t="inlineStr">
         <is>
-          <t>410000.00</t>
+          <t>350000.00</t>
         </is>
       </c>
       <c r="Z30" s="0" t="inlineStr">
@@ -1140,7 +1140,7 @@
       </c>
       <c r="X31" s="0" t="inlineStr">
         <is>
-          <t>637000.00</t>
+          <t>267000.00</t>
         </is>
       </c>
       <c r="Z31" s="0" t="inlineStr">
@@ -1556,7 +1556,7 @@
       </c>
       <c r="X44" s="0" t="inlineStr">
         <is>
-          <t>408000.00</t>
+          <t>68000.00</t>
         </is>
       </c>
       <c r="Z44" s="0" t="inlineStr">
@@ -1716,7 +1716,7 @@
       </c>
       <c r="X49" s="0" t="inlineStr">
         <is>
-          <t>1020000.00</t>
+          <t>684000.00</t>
         </is>
       </c>
       <c r="Z49" s="0" t="inlineStr">
@@ -1812,7 +1812,7 @@
       </c>
       <c r="X52" s="0" t="inlineStr">
         <is>
-          <t>1198000.00</t>
+          <t>730000.00</t>
         </is>
       </c>
       <c r="Z52" s="0" t="inlineStr">

</xml_diff>

<commit_message>
Reapply "Add OpenRouter API To GPT LLM for query"
This reverts commit 0ab6aafe410989b77a9221ffde15ed0c33e8dc3b.
</commit_message>
<xml_diff>
--- a/Excels/customers_export.xlsx
+++ b/Excels/customers_export.xlsx
@@ -212,7 +212,7 @@
       </c>
       <c r="X2" s="0" t="inlineStr">
         <is>
-          <t>537000.00</t>
+          <t>1640000.00</t>
         </is>
       </c>
       <c r="Z2" s="0" t="inlineStr">
@@ -244,7 +244,7 @@
       </c>
       <c r="X3" s="0" t="inlineStr">
         <is>
-          <t>1876100.00</t>
+          <t>1944100.00</t>
         </is>
       </c>
       <c r="Z3" s="0" t="inlineStr">
@@ -308,7 +308,7 @@
       </c>
       <c r="X5" s="0" t="inlineStr">
         <is>
-          <t>957500.00</t>
+          <t>1743500.00</t>
         </is>
       </c>
       <c r="Z5" s="0" t="inlineStr">
@@ -340,7 +340,7 @@
       </c>
       <c r="X6" s="0" t="inlineStr">
         <is>
-          <t>2014500.00</t>
+          <t>2895000.00</t>
         </is>
       </c>
       <c r="Z6" s="0" t="inlineStr">
@@ -404,7 +404,7 @@
       </c>
       <c r="X8" s="0" t="inlineStr">
         <is>
-          <t>345500.00</t>
+          <t>0.00</t>
         </is>
       </c>
       <c r="Z8" s="0" t="inlineStr">
@@ -500,7 +500,7 @@
       </c>
       <c r="X11" s="0" t="inlineStr">
         <is>
-          <t>1597000.00</t>
+          <t>1477000.00</t>
         </is>
       </c>
       <c r="Z11" s="0" t="inlineStr">
@@ -532,7 +532,7 @@
       </c>
       <c r="X12" s="0" t="inlineStr">
         <is>
-          <t>16364300.00</t>
+          <t>29980500.00</t>
         </is>
       </c>
       <c r="Z12" s="0" t="inlineStr">
@@ -884,7 +884,7 @@
       </c>
       <c r="X23" s="0" t="inlineStr">
         <is>
-          <t>796000.00</t>
+          <t>1941000.00</t>
         </is>
       </c>
       <c r="Z23" s="0" t="inlineStr">
@@ -916,7 +916,7 @@
       </c>
       <c r="X24" s="0" t="inlineStr">
         <is>
-          <t>1533000.00</t>
+          <t>2526000.00</t>
         </is>
       </c>
       <c r="Z24" s="0" t="inlineStr">
@@ -1044,7 +1044,7 @@
       </c>
       <c r="X28" s="0" t="inlineStr">
         <is>
-          <t>1341000.00</t>
+          <t>1778000.00</t>
         </is>
       </c>
       <c r="Z28" s="0" t="inlineStr">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="X29" s="0" t="inlineStr">
         <is>
-          <t>263000.00</t>
+          <t>653000.00</t>
         </is>
       </c>
       <c r="Z29" s="0" t="inlineStr">
@@ -1108,7 +1108,7 @@
       </c>
       <c r="X30" s="0" t="inlineStr">
         <is>
-          <t>350000.00</t>
+          <t>410000.00</t>
         </is>
       </c>
       <c r="Z30" s="0" t="inlineStr">
@@ -1140,7 +1140,7 @@
       </c>
       <c r="X31" s="0" t="inlineStr">
         <is>
-          <t>267000.00</t>
+          <t>637000.00</t>
         </is>
       </c>
       <c r="Z31" s="0" t="inlineStr">
@@ -1556,7 +1556,7 @@
       </c>
       <c r="X44" s="0" t="inlineStr">
         <is>
-          <t>68000.00</t>
+          <t>408000.00</t>
         </is>
       </c>
       <c r="Z44" s="0" t="inlineStr">
@@ -1716,7 +1716,7 @@
       </c>
       <c r="X49" s="0" t="inlineStr">
         <is>
-          <t>684000.00</t>
+          <t>1020000.00</t>
         </is>
       </c>
       <c r="Z49" s="0" t="inlineStr">
@@ -1812,7 +1812,7 @@
       </c>
       <c r="X52" s="0" t="inlineStr">
         <is>
-          <t>730000.00</t>
+          <t>1198000.00</t>
         </is>
       </c>
       <c r="Z52" s="0" t="inlineStr">

</xml_diff>